<commit_message>
chore: repopulate CESO and APHIS user collections from updated Excel, fix admin upload script for service account path
</commit_message>
<xml_diff>
--- a/BASES DATOS/usuarios_consolidados.xlsx
+++ b/BASES DATOS/usuarios_consolidados.xlsx
@@ -14,11 +14,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="81">
   <si>
     <t>nombre</t>
   </si>
   <si>
+    <t>cargo</t>
+  </si>
+  <si>
+    <t>dependencia</t>
+  </si>
+  <si>
+    <t>telefono</t>
+  </si>
+  <si>
     <t>correo</t>
   </si>
   <si>
@@ -37,6 +46,12 @@
     <t>Jorge Carlos Berlín Montero</t>
   </si>
   <si>
+    <t>Representante Estatal</t>
+  </si>
+  <si>
+    <t>SADER</t>
+  </si>
+  <si>
     <t>representacion.yuc@agricultura.gob.mx</t>
   </si>
   <si>
@@ -49,9 +64,15 @@
     <t>CESO,APHIS</t>
   </si>
   <si>
+    <t>view,download,upload,edit</t>
+  </si>
+  <si>
     <t>Abigail Estrada Estrada</t>
   </si>
   <si>
+    <t>Subdelegado Agropecuario</t>
+  </si>
+  <si>
     <t>abigail.estrada@yct.agricultura.gob.mx</t>
   </si>
   <si>
@@ -61,6 +82,9 @@
     <t>Luis Martín Flores Martínez</t>
   </si>
   <si>
+    <t>Jefe de Programa de Fomento Agropecuario</t>
+  </si>
+  <si>
     <t>luis.floresm@yct.agricultura.gob.mx</t>
   </si>
   <si>
@@ -70,6 +94,9 @@
     <t>Sergio Muñoz de Alba Medrano</t>
   </si>
   <si>
+    <t>PSI Independiente</t>
+  </si>
+  <si>
     <t>smunoz.sader@gmail.com</t>
   </si>
   <si>
@@ -79,9 +106,18 @@
     <t>MunozSader#99</t>
   </si>
   <si>
+    <t>view,download,upload,edit,admin</t>
+  </si>
+  <si>
     <t>Juan Carlos Rodríguez Andrade</t>
   </si>
   <si>
+    <t>Director de Sanidad</t>
+  </si>
+  <si>
+    <t>SEDER</t>
+  </si>
+  <si>
     <t>juan.rodrigueza@yucatan.gob.mx</t>
   </si>
   <si>
@@ -94,6 +130,9 @@
     <t>Moisés Abraham Martín Sima</t>
   </si>
   <si>
+    <t>Jefe de Campañas</t>
+  </si>
+  <si>
     <t>moises.martin@yucatan.gob.mx</t>
   </si>
   <si>
@@ -103,6 +142,9 @@
     <t>José Joaquín Peral Rodríguez</t>
   </si>
   <si>
+    <t>SENASICA</t>
+  </si>
+  <si>
     <t>jose.peral@senasica.gob.mx</t>
   </si>
   <si>
@@ -121,6 +163,12 @@
     <t>Roger Armando Díaz Mendoza</t>
   </si>
   <si>
+    <t>Presidente Comité</t>
+  </si>
+  <si>
+    <t>CFYPPF</t>
+  </si>
+  <si>
     <t>ad1609@hotmail.com</t>
   </si>
   <si>
@@ -133,13 +181,22 @@
     <t>Alfredo Colín Álvarez</t>
   </si>
   <si>
+    <t xml:space="preserve">Gerente Comité </t>
+  </si>
+  <si>
     <t>efppygerente@gmail.com</t>
   </si>
   <si>
     <t>CefppyGer@789</t>
   </si>
   <si>
-    <t>Francis A. Genovés Chanona</t>
+    <t>Francis A. Genovéz Chanona</t>
+  </si>
+  <si>
+    <t>Gerente Regional</t>
+  </si>
+  <si>
+    <t>SINIIGA</t>
   </si>
   <si>
     <t>francis.genoves@siniiga.gob.mx</t>
@@ -151,36 +208,18 @@
     <t>Siniiga2025!</t>
   </si>
   <si>
-    <t xml:space="preserve">Gerardo Solís Pasos </t>
-  </si>
-  <si>
-    <t>gerardo.solis@yucatan.gob.mx</t>
-  </si>
-  <si>
-    <t>SederYucSOLIS@2024</t>
+    <t>Jorge Carlos Concha Cutz</t>
+  </si>
+  <si>
+    <t>jorgeconcha_75@hotmail.com</t>
+  </si>
+  <si>
+    <t>ConchaCefppy$3</t>
   </si>
   <si>
     <t>APHIS</t>
   </si>
   <si>
-    <t>Jorge Carlos Concha Cutz</t>
-  </si>
-  <si>
-    <t>jorgeconcha_75@hotmail.com</t>
-  </si>
-  <si>
-    <t>ConchaCefppy$3</t>
-  </si>
-  <si>
-    <t>Noé J. Cepeda Lizama</t>
-  </si>
-  <si>
-    <t>noe.cepeda@ugroy.org</t>
-  </si>
-  <si>
-    <t>UgroyNoe$456</t>
-  </si>
-  <si>
     <t>Oscar Correa</t>
   </si>
   <si>
@@ -190,13 +229,34 @@
     <t>CorreaCefppy#7</t>
   </si>
   <si>
-    <t>Ivonne Galera Chan</t>
-  </si>
-  <si>
-    <t>ivonne.galera@vas.org</t>
-  </si>
-  <si>
-    <t>VasGalera$123</t>
+    <t>Angel Miqueas Castillo Caamal</t>
+  </si>
+  <si>
+    <t>Jefe Ventanilla UGRY</t>
+  </si>
+  <si>
+    <t>UGRY</t>
+  </si>
+  <si>
+    <t>vas.yuc@ventanillasiniiga.org.mx</t>
+  </si>
+  <si>
+    <t>MiqueasUgRy#5</t>
+  </si>
+  <si>
+    <t>CESO</t>
+  </si>
+  <si>
+    <t>Edgardo Gilberto Medina Estrada</t>
+  </si>
+  <si>
+    <t>Secretario</t>
+  </si>
+  <si>
+    <t>edgardo.medinar@yucatan.gob.mx</t>
+  </si>
+  <si>
+    <t>SederYuc01@2025</t>
   </si>
 </sst>
 </file>
@@ -204,13 +264,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -221,7 +287,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -233,13 +306,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -543,15 +625,18 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="26.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="28.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="24.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="31.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="19.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="37.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -564,7 +649,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -573,294 +658,448 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="D2" s="3">
+        <v>9991551508</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1"/>
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3">
+        <v>9933045348</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2461113005</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="1"/>
+      <c r="I4" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
+      </c>
+      <c r="D5" s="3">
+        <v>9992005550</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>24</v>
+        <v>33</v>
+      </c>
+      <c r="D6" s="3">
+        <v>9991852636</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="1"/>
+        <v>34</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
+      </c>
+      <c r="D7" s="3">
+        <v>9911003936</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="1"/>
+        <v>39</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="3">
+        <v>9993227938</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>33</v>
+        <v>42</v>
+      </c>
+      <c r="D9" s="3">
+        <v>9991277762</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>37</v>
+        <v>50</v>
+      </c>
+      <c r="D10" s="3">
+        <v>9992422545</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>40</v>
+        <v>50</v>
+      </c>
+      <c r="D11" s="3">
+        <v>9994236678</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="1"/>
+        <v>56</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
+      </c>
+      <c r="D12" s="3">
+        <v>9616089724</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="1"/>
+        <v>61</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
+      </c>
+      <c r="D13" s="3">
+        <v>9911024277</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" s="1"/>
+        <v>65</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="D14" s="2"/>
       <c r="E14" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="1"/>
+        <v>69</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>54</v>
+        <v>73</v>
+      </c>
+      <c r="D15" s="3">
+        <v>9994045018</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="1"/>
+        <v>74</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>57</v>
+        <v>33</v>
+      </c>
+      <c r="D16" s="3">
+        <v>9992246695</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F17" s="1"/>
+        <v>79</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>